<commit_message>
flying-swarm: spreadsheet landscape fit-to-width for clean printing/PDF
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/flying-swarm/engineering/swarm-drone-calcs.xlsx
+++ b/examples/flying-swarm/engineering/swarm-drone-calcs.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Motor-Weight-Power" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Motor-Weight-Power'!$A$1:$D$46</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -521,7 +523,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1164,5 +1166,6 @@
     <mergeCell ref="A42:D42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>